<commit_message>
week 6 query strings generated.
</commit_message>
<xml_diff>
--- a/Function 3/evals.xlsx
+++ b/Function 3/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96025F5A-9DEC-4F1E-A1F5-4FE65C376CDF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA072E0-C5DD-4B69-9046-763668E98768}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -519,10 +519,10 @@
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="3"/>
       <c r="D8" s="2">
         <v>1</v>
       </c>
@@ -626,55 +626,6 @@
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="H14:I14"/>
@@ -691,6 +642,55 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="J5:K5"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J9:K9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>